<commit_message>
code added for percentage calculation
</commit_message>
<xml_diff>
--- a/uploads/gender_biased_words.xlsx
+++ b/uploads/gender_biased_words.xlsx
@@ -1,39 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\DIAWorkspace\DIA\uploads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9597DB9-FD47-460E-9F13-1CB2F3C47606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="19425" windowHeight="10425"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="word" sheetId="1" r:id="rId1"/>
+    <sheet name="Words" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>word</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
   <si>
     <t>he</t>
   </si>
@@ -56,13 +48,22 @@
     <t>she</t>
   </si>
   <si>
-    <t>woman</t>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Words</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Female</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -154,7 +155,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -189,7 +190,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -366,60 +367,79 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>